<commit_message>
fix: assign personal reference support multiple people in a sheet
</commit_message>
<xml_diff>
--- a/tables_filled/22b5da6f-d542-421f-b00b-8d360f06d0b0.xlsx
+++ b/tables_filled/22b5da6f-d542-421f-b00b-8d360f06d0b0.xlsx
@@ -2767,7 +2767,7 @@
       </c>
       <c r="C9" s="76" t="inlineStr">
         <is>
-          <t>TA-1</t>
+          <t>Referenz 1</t>
         </is>
       </c>
       <c r="D9" s="77" t="inlineStr">
@@ -2818,7 +2818,7 @@
       </c>
       <c r="C11" s="116" t="inlineStr">
         <is>
-          <t>Universitätsklinikum Schleswig-Holstein AöR</t>
+          <t>Sanierung und Umbau Klinikgebäude Haus C, Universitätsklinikum Schleswig-Holstein AöR</t>
         </is>
       </c>
       <c r="D11" s="116" t="inlineStr">
@@ -2892,7 +2892,7 @@
       </c>
       <c r="E14" s="116" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>Ja</t>
         </is>
       </c>
     </row>
@@ -2972,7 +2972,7 @@
       </c>
       <c r="E17" s="116" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Hamburg, Germany</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="C18" s="116" t="inlineStr">
         <is>
-          <t>Februar 2024</t>
+          <t>February 2024</t>
         </is>
       </c>
       <c r="D18" s="72" t="inlineStr">
@@ -3001,7 +3001,7 @@
       </c>
       <c r="E18" s="116" t="inlineStr">
         <is>
-          <t>Juni 2019</t>
+          <t>June 2019</t>
         </is>
       </c>
     </row>
@@ -19524,7 +19524,7 @@
       </c>
       <c r="E24" s="116" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>Ja</t>
         </is>
       </c>
     </row>
@@ -19551,7 +19551,7 @@
       </c>
       <c r="E25" s="116" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>Ja</t>
         </is>
       </c>
     </row>
@@ -35983,7 +35983,7 @@
       </c>
       <c r="E27" s="116" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>Ja</t>
         </is>
       </c>
     </row>

</xml_diff>